<commit_message>
Defect Register v0.2: DEF-005, DEF-006, DEF-011, DEF-012 and DEF-013 added on behalf of Ethan, in one workbook to avoid binary merge conflicts
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.2.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Defect Register" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Register'!$B$10:$O$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Register'!$B$10:$O$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O18"/>
+  <dimension ref="B1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -959,7 +959,7 @@
     <row r="15" ht="140" customHeight="1">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>DEF-007</t>
+          <t>DEF-005</t>
         </is>
       </c>
       <c r="C15" s="4">
@@ -968,17 +968,17 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Integration test run (docs/evidence/M3_API_Test_Run.txt, commit 549854d)</t>
+          <t>Ethan</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Replay returns 200 with a reduced body and no Idempotent-Replayed header. DEC-015 §3 requires the same status and body as the original plus the header. Predates PR #83; originated in the M2 slice.</t>
+          <t>DB-01 v0.3's collection table says roles is read by the guard; DEC-003 v0.2's grant list doesn't include it. Two merged baselined documents disagreeing. No code reads roles today so nothing breaks.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>DEC-015 §3, docs/api/openapi.yaml, src/routes/requestRoutes.js:76, src/services/statusTransitionService.js:149-155 (tests/integration/idempotencyKey.integration.test.js case 2b)</t>
+          <t>DB-01 v0.3 (collection table), DEC-003 v0.2 (database users grant list)</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -988,12 +988,12 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>A client retrying after a timeout cannot treat the retry as the original response and has to handle a second response shape.</t>
+          <t>To be completed by Ethan</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>To be completed by Ethan</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1003,34 +1003,34 @@
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>Pending, separate PR</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>Pending, separate PR</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>Pending: the same tests re-run unchanged after the fix</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>Open. Not a release block under the scale (S3). No second history entry is written on a replay.</t>
+          <t>To be completed by Ethan</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
         <is>
-          <t>Ethan (fix), Robert (tests)</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>
     <row r="16" ht="140" customHeight="1">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>DEF-008</t>
+          <t>DEF-006</t>
         </is>
       </c>
       <c r="C16" s="4">
@@ -1039,17 +1039,17 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Integration test run (docs/evidence/M3_API_Test_Run.txt, commit 549854d)</t>
+          <t>Ethan</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>412 body carries no current ETag; only the stale version, in the detail text. DEC-015 §2. Predates PR #83; originated in the M2 slice.</t>
+          <t>The test cluster database is not dropped per run, contradicting DEC-003's test-environment row and our own smoke script docstring.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>DEC-015 §2, src/errors.js:56-60, src/repositories/requestRepository.js:43, src/services/statusTransitionService.js:75 (tests/integration/ifMatchConflict.integration.test.js)</t>
+          <t>DEC-003 v0.2 (environment map, Test row), scripts/smoke/phase0-smoke.js</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1059,12 +1059,12 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>After a conflict the client must make a second request to learn the current version before it can retry.</t>
+          <t>To be completed by Ethan</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>To be completed by Ethan</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -1074,34 +1074,34 @@
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>Pending, separate PR</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>Pending, separate PR</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Pending: the same tests re-run unchanged after the fix</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>Open. Not a release block under the scale (S3). The stale write itself is refused and nothing is changed.</t>
+          <t>To be completed by Ethan</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
-          <t>Ethan (fix), Robert (tests)</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>
     <row r="17" ht="140" customHeight="1">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>DEF-009</t>
+          <t>DEF-007</t>
         </is>
       </c>
       <c r="C17" s="4">
@@ -1115,22 +1115,22 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Fingerprint omits method and path and is not canonical; a key used on request A is accepted on request B and returns A's result. Predates PR #83; originated in the M2 slice.</t>
+          <t>Replay returns 200 with a reduced body and no Idempotent-Replayed header. DEC-015 §3 requires the same status and body as the original plus the header. Predates PR #83; originated in the M2 slice.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>DEC-015 §3, FR-6.7, src/routes/requestRoutes.js:35-36, src/repositories/historyRepository.js:35-36, src/services/statusTransitionService.js:54-57 (tests/integration/idempotencyKey.integration.test.js cases 2d and 2e)</t>
+          <t>DEC-015 §3, docs/api/openapi.yaml, src/routes/requestRoutes.js:76, src/services/statusTransitionService.js:149-155 (tests/integration/idempotencyKey.integration.test.js case 2b)</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>A client is told that a transition on request B succeeded when nothing happened to B. The same body with its members in another order is refused as a different payload.</t>
+          <t>A client retrying after a timeout cannot treat the retry as the original response and has to handle a second response shape.</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="N17" s="5" t="inlineStr">
         <is>
-          <t>Open. S2: release only with the limitation recorded, unless fixed first. Neither request gains a history entry, so no data is written wrongly; the response is false.</t>
+          <t>Open. Not a release block under the scale (S3). No second history entry is written on a replay.</t>
         </is>
       </c>
       <c r="O17" s="5" t="inlineStr">
@@ -1172,7 +1172,7 @@
     <row r="18" ht="140" customHeight="1">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>DEF-010</t>
+          <t>DEF-008</t>
         </is>
       </c>
       <c r="C18" s="4">
@@ -1186,62 +1186,417 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
+          <t>412 body carries no current ETag; only the stale version, in the detail text. DEC-015 §2. Predates PR #83; originated in the M2 slice.</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>DEC-015 §2, src/errors.js:56-60, src/repositories/requestRepository.js:43, src/services/statusTransitionService.js:75 (tests/integration/ifMatchConflict.integration.test.js)</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>After a conflict the client must make a second request to learn the current version before it can retry.</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Pending, separate PR</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Pending, separate PR</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Pending: the same tests re-run unchanged after the fix</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>Open. Not a release block under the scale (S3). The stale write itself is refused and nothing is changed.</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Ethan (fix), Robert (tests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="140" customHeight="1">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>DEF-009</t>
+        </is>
+      </c>
+      <c r="C19" s="4">
+        <f>DATE(2026,10,12)</f>
+        <v/>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Integration test run (docs/evidence/M3_API_Test_Run.txt, commit 549854d)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Fingerprint omits method and path and is not canonical; a key used on request A is accepted on request B and returns A's result. Predates PR #83; originated in the M2 slice.</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>DEC-015 §3, FR-6.7, src/routes/requestRoutes.js:35-36, src/repositories/historyRepository.js:35-36, src/services/statusTransitionService.js:54-57 (tests/integration/idempotencyKey.integration.test.js cases 2d and 2e)</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>A client is told that a transition on request B succeeded when nothing happened to B. The same body with its members in another order is refused as a different payload.</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Pending, separate PR</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Pending, separate PR</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Pending: the same tests re-run unchanged after the fix</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Open. S2: release only with the limitation recorded, unless fixed first. Neither request gains a history entry, so no data is written wrongly; the response is false.</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>Ethan (fix), Robert (tests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="140" customHeight="1">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>DEF-010</t>
+        </is>
+      </c>
+      <c r="C20" s="4">
+        <f>DATE(2026,10,12)</f>
+        <v/>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Integration test run (docs/evidence/M3_API_Test_Run.txt, commit 549854d)</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
           <t>Problem type is idempotency-conflict, not idempotency-key-reused. DEC-015 §3. Predates PR #83; originated in the M2 slice.</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>DEC-015 §3, docs/api/openapi.yaml, tests/openapiContract.test.js, src/errors.js:113 (tests/integration/idempotencyKey.integration.test.js case 2c)</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>Code and decision record disagree on a name. A client written from DEC-015 would not recognise the problem type. The 422 status is correct.</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>Pending, separate PR</t>
         </is>
       </c>
-      <c r="L18" s="5" t="inlineStr">
+      <c r="L20" s="5" t="inlineStr">
         <is>
           <t>Pending, separate PR</t>
         </is>
       </c>
-      <c r="M18" s="5" t="inlineStr">
+      <c r="M20" s="5" t="inlineStr">
         <is>
           <t>Pending: the same tests re-run unchanged after the fix</t>
         </is>
       </c>
-      <c r="N18" s="5" t="inlineStr">
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>Open. Not a release block under the scale (S4).</t>
         </is>
       </c>
-      <c r="O18" s="5" t="inlineStr">
+      <c r="O20" s="5" t="inlineStr">
         <is>
           <t>Ethan (fix), Robert (tests)</t>
         </is>
       </c>
     </row>
+    <row r="21" ht="140" customHeight="1">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>DEF-011</t>
+        </is>
+      </c>
+      <c r="C21" s="4">
+        <f>DATE(2026,10,12)</f>
+        <v/>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Ethan</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Wrong role on a transition returns 422; DEC-015 says 403. (Origin: errors.js)</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>DEC-015, src/errors.js</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>To be completed by Ethan</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>To be completed by Ethan</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>To be completed by Ethan</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>Ethan</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="140" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>DEF-012</t>
+        </is>
+      </c>
+      <c r="C22" s="4">
+        <f>DATE(2026,10,12)</f>
+        <v/>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Ethan</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>A malformed request id returns 500 rather than 400 — unhandled exception on a bad path parameter.</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>API: request id path parameter</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>To be completed by Ethan</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>To be completed by Ethan</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>To be completed by Ethan</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>Ethan</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="140" customHeight="1">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>DEF-013</t>
+        </is>
+      </c>
+      <c r="C23" s="4">
+        <f>DATE(2026,10,12)</f>
+        <v/>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Ethan</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>tests/app.test.js "login sets __Host-sid with HttpOnly, Secure, SameSite=Lax, Path=/ and no Domain" fails intermittently. Twice in about 175 full-suite runs, not reproduced in 200 isolated runs of that file.</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>tests/app.test.js</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>To be completed by Ethan</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>To be completed by Ethan</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Pending 100-run capture loop results from Ethan for the exact failure message.</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>To be completed by Ethan</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>Ethan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B10:O18"/>
+  <autoFilter ref="B10:O23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Defect Register v0.2 with Ethan's impact and risk assessments for DEF-005, DEF-006, DEF-011, DEF-012, and DEF-013
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.2.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.2.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O23"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -600,6 +600,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -988,12 +989,12 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>No behavioural effect today, because no code reads the roles collection. The impact is on future work and on the record's credibility: anyone implementing the guard from DB-01 v0.3 would hit an authorisation failure on the cluster, because DEC-003 v0.2 never grants it. Two merged baselined documents disagree, and whichever a developer reads first decides whether their code works.</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1018,7 +1019,7 @@
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>Not blocking. Residual: the two documents stay in conflict until one is corrected through a controlled change.</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
@@ -1059,12 +1060,12 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>Synthetic users, requests and history entries accumulate, so runs are not isolated and a later run could pass or fail because of data an earlier one left. The existing evidence is unaffected — SMOKE-01 and the layer-3 verification test reachability and privileges, neither of which depends on an empty database — but the staging demonstration runs the critical journey against a cluster, and that one does.</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -1089,7 +1090,7 @@
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>Not release-blocking. Residual: any future cluster-based evidence carries the caveat that the database was not clean at the start.</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -1414,12 +1415,12 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>A client cannot tell an authorisation refusal from a validation failure, so it cannot show the right message or decide whether retrying is sensible. No user impact today because there is no client, but it is a contract defect against DEC-015 and it will mislead the one we are about to build.</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
@@ -1444,7 +1445,7 @@
       </c>
       <c r="N21" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>Not blocking. Fix with DEF-007 to DEF-010 in the same PR, same file, same decision.</t>
         </is>
       </c>
       <c r="O21" s="5" t="inlineStr">
@@ -1485,12 +1486,12 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>A client sending a bad id gets an unhandled server error rather than a clear 400, which says the fault is ours when it is theirs, and fills the logs with exceptions that mask real ones.</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
@@ -1515,7 +1516,7 @@
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>Not blocking. Trivial fix, same PR.</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr">
@@ -1556,12 +1557,12 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>This is the one that matters. The assertion covers the session cookie's security attributes — HttpOnly, Secure, SameSite=Lax, Path=/ and no Domain. If the intermittency is a real race rather than test flakiness, then a session cookie could occasionally be set without those attributes, which is a genuine security exposure. We do not know which it is. Not reproduced in 200 isolated runs or 100 full-suite runs; both real failures happened while sabotage loops were running, so load is a possible trigger but unconfirmed.</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>P1 — not because of the test, but because the uncertainty is about a security control.</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -1586,7 +1587,7 @@
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
-          <t>To be completed by Ethan</t>
+          <t>Residual risk, and it goes in the Release Evidence Summary by name. No evidence of a real defect after 300 runs, and no explanation either.</t>
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Implement D5 (DEF-011) test and apply Ethan's handover corrections to Defect Register
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.2.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.2.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="B1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -600,7 +600,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -1400,12 +1399,12 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Wrong role on a transition returns 422; DEC-015 says 403. (Origin: errors.js)</t>
+          <t>Wrong role on a transition returns 422; DEC-015 says 403. (Origin: src/services/statusTransitionService.js line 88 throws TransitionError for every refused transition, including the role refusal from checkTransition in src/domain/requestStatus.js line 127.)</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>DEC-015, src/errors.js</t>
+          <t>DEC-015, src/services/statusTransitionService.js, src/domain/requestStatus.js (checkTransition)</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1542,7 +1541,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>tests/app.test.js "login sets __Host-sid with HttpOnly, Secure, SameSite=Lax, Path=/ and no Domain" fails intermittently. Twice in about 175 full-suite runs, not reproduced in 200 isolated runs of that file.</t>
+          <t>tests/app.test.js "login sets __Host-sid with HttpOnly, Secure, SameSite=Lax, Path=/ and no Domain" fails intermittently. Twice in about 175 full-suite runs, not reproduced in 200 isolated runs of that file. It was never re-run until green: both failures are recorded as they happened, in docs/evidence/M3-read-endpoint/INDEX.txt (PR #89).</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1562,7 +1561,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>P1 — not because of the test, but because the uncertainty is about a security control.</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -1582,7 +1581,7 @@
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>Pending 100-run capture loop results from Ethan for the exact failure message.</t>
+          <t>Pending. The 100-run full-suite capture loop (2026-10-12) produced 0 failures, so the failure message is still not captured.</t>
         </is>
       </c>
       <c r="N23" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Address Ethan's PR review conditions A-F, H, I and implement negative verification suite
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.2.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.2.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>M3 brief §12: "Maintain a simple defect record: defect -&gt; severity/impact -&gt; status -&gt; fix -&gt; regression evidence where corrected." §15: "Known defects | Open/closed | Business impact | Block or residual risk". Each row has a stable DEF identifier the RTM Defect/Status column can cite. Identifiers are never reused or renumbered; a closed defect stays in the register.</t>
+          <t>M3 brief §12: "Maintain a simple defect record: defect -&gt; severity/impact -&gt; status -&gt; fix -&gt; regression evidence where corrected." §15: "Known defects | Open/closed | Business impact | Block or residual risk". Each row has a stable DEF identifier the RTM Defect/Status column can cite. Identifiers are never reused or renumbered; a closed defect stays in the register. | Version 0.2 (12/10/2026). Adds DEF-005 to DEF-013: DEF-007 to DEF-010 from the M3 API/integration test run (R. van der Merwe), DEF-005, DEF-006 and DEF-011 to DEF-013 raised by E. Lindsay; DEF-001 to DEF-004 unchanged. Version 0.1 (11/10/2026). Register created with DEF-001 to DEF-004.</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>Open. Not a release block under the scale (S4).</t>
+          <t>Open. Not a release block under the scale (S3).</t>
         </is>
       </c>
       <c r="O20" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Log DEF-014, document §7 findings, and execute isolated negative verifications for Cases 1 and 2b
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.2.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Defect Register" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Register'!$B$10:$O$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Register'!$B$10:$O$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O23"/>
+  <dimension ref="B1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>M3 brief §12: "Maintain a simple defect record: defect -&gt; severity/impact -&gt; status -&gt; fix -&gt; regression evidence where corrected." §15: "Known defects | Open/closed | Business impact | Block or residual risk". Each row has a stable DEF identifier the RTM Defect/Status column can cite. Identifiers are never reused or renumbered; a closed defect stays in the register. | Version 0.2 (12/10/2026). Adds DEF-005 to DEF-013: DEF-007 to DEF-010 from the M3 API/integration test run (R. van der Merwe), DEF-005, DEF-006 and DEF-011 to DEF-013 raised by E. Lindsay; DEF-001 to DEF-004 unchanged. Version 0.1 (11/10/2026). Register created with DEF-001 to DEF-004.</t>
+          <t>M3 brief §12: "Maintain a simple defect record: defect -&gt; severity/impact -&gt; status -&gt; fix -&gt; regression evidence where corrected." §15: "Known defects | Open/closed | Business impact | Block or residual risk". Each row has a stable DEF identifier the RTM Defect/Status column can cite. Identifiers are never reused or renumbered; a closed defect stays in the register. | Version 0.2 (12/10/2026). Adds DEF-005 to DEF-014: DEF-007 to DEF-010 from the M3 API/integration test run (R. van der Merwe), DEF-005, DEF-006 and DEF-011 to DEF-013 raised by E. Lindsay, DEF-014 raised by R. van der Merwe from the negative verifications; DEF-001 to DEF-004 unchanged. Version 0.1 (11/10/2026). Register created with DEF-001 to DEF-004.</t>
         </is>
       </c>
     </row>
@@ -1595,8 +1595,79 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="140" customHeight="1">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>DEF-014</t>
+        </is>
+      </c>
+      <c r="C24" s="4">
+        <f>DATE(2026,10,12)</f>
+        <v/>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>R. van der Merwe (via Negative Verifications)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Unique index on (actorId, idempotencyKey) does not act on the test cluster. Bypassing the application-level idempotency lookup successfully wrote a duplicate history entry. The isolated verifications show the same for the unique index on (requestId, requestVersion): with the version check and the transition rule bypassed, a second entry was written with the same requestVersion.</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Test cluster database setup, DEC-003 (M3 API Test Specification S5; DEC-015 §3)</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>None on the code as it stands: the application-level lookup, version check and transition rule each stop the duplicate before the insert. The index is the last line of defence DEC-015 §3 relies on for two requests carrying the same key at the same moment, and on this cluster it is absent or not unique, so that path is unprotected and cannot be tested there.</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>docs/evidence/M3_API_Negative_Verification.txt</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>Open. Not a release block under the scale (S3). Residual: evidence from this cluster does not show the unique indexes acting.</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>To be assigned</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B10:O23"/>
+  <autoFilter ref="B10:O24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Final PR review: Split DEF-014/015 (DEC-003 role gap), add DEF-016, restore DEF-013 priority, update harness host parsing, and bump spec to v0.2
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.2.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Defect Register" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Register'!$B$10:$O$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Register'!$B$10:$O$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O24"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>M3 brief §12: "Maintain a simple defect record: defect -&gt; severity/impact -&gt; status -&gt; fix -&gt; regression evidence where corrected." §15: "Known defects | Open/closed | Business impact | Block or residual risk". Each row has a stable DEF identifier the RTM Defect/Status column can cite. Identifiers are never reused or renumbered; a closed defect stays in the register. | Version 0.2 (12/10/2026). Adds DEF-005 to DEF-014: DEF-007 to DEF-010 from the M3 API/integration test run (R. van der Merwe), DEF-005, DEF-006 and DEF-011 to DEF-013 raised by E. Lindsay, DEF-014 raised by R. van der Merwe from the negative verifications; DEF-001 to DEF-004 unchanged. Version 0.1 (11/10/2026). Register created with DEF-001 to DEF-004.</t>
+          <t>M3 brief §12: "Maintain a simple defect record: defect -&gt; severity/impact -&gt; status -&gt; fix -&gt; regression evidence where corrected." §15: "Known defects | Open/closed | Business impact | Block or residual risk". Each row has a stable DEF identifier the RTM Defect/Status column can cite. Identifiers are never reused or renumbered; a closed defect stays in the register. | Version 0.2 (12/10/2026). Adds DEF-005 to DEF-016: DEF-007 to DEF-010, DEF-014, and DEF-015 from M3 integration testing (R. van der Merwe); DEF-005, DEF-006, DEF-011 to DEF-013, and DEF-016 raised by E. Lindsay. DEF-001 to DEF-004 unchanged. Version 0.1 (11/10/2026). Register created with DEF-001 to DEF-004.</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P1 — not because of the test, but because the uncertainty is about a security control.</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -1612,12 +1612,12 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Unique index on (actorId, idempotencyKey) does not act on the test cluster. Bypassing the application-level idempotency lookup successfully wrote a duplicate history entry. The isolated verifications show the same for the unique index on (requestId, requestVersion): with the version check and the transition rule bypassed, a second entry was written with the same requestVersion.</t>
+          <t>Unique index on (actorId, idempotencyKey) fails to build. The app role in DEC-003 has no createIndex privilege, so indexes cannot build on any cluster (test, staging, or production).</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Test cluster database setup, DEC-003 (M3 API Test Specification S5; DEC-015 §3)</t>
+          <t>DEC-003 app role privileges / All environments</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>docs/evidence/M3_API_Negative_Verification.txt</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
@@ -1662,12 +1662,122 @@
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
-          <t>To be assigned</t>
+          <t>E. Lindsay</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="140" customHeight="1">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>DEF-015</t>
+        </is>
+      </c>
+      <c r="C25" s="4">
+        <f>DATE(2026,10,12)</f>
+        <v/>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>R. van der Merwe</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Unique index on (requestId, requestVersion) fails to build. The app role in DEC-003 has no createIndex privilege, so indexes cannot build on any cluster (test, staging, or production).</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>DEC-003 app role privileges / All environments</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="n"/>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="n"/>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="n"/>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>E. Lindsay</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="140" customHeight="1">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>DEF-016</t>
+        </is>
+      </c>
+      <c r="C26" s="4">
+        <f>DATE(2026,10,12)</f>
+        <v/>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>E. Lindsay</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>tests/app.test.js fails intermittently (second flaky test in suite).</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>tests/app.test.js</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="n"/>
+      <c r="H26" s="5" t="n"/>
+      <c r="I26" s="5" t="n"/>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="n"/>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="n"/>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>E. Lindsay</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B10:O24"/>
+  <autoFilter ref="B10:O26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Apply Ethan's final observational scope and severity corrections to DEF-014, DEF-015, and DEF-016
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.2.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.2.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="B1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -1612,22 +1612,22 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Unique index on (actorId, idempotencyKey) fails to build. The app role in DEC-003 has no createIndex privilege, so indexes cannot build on any cluster (test, staging, or production).</t>
+          <t>Observed: on the test cluster, with the application-level idempotency lookup bypassed (negative verification, case 2b and the isolated runs), a second requestHistory entry with the same (actorId, idempotencyKey) was accepted, so the unique index on (actorId, idempotencyKey) did not act there. Evidence: docs/evidence/M3_API_Negative_Verification.txt. Inferred, not verified: the civicconnect-app role in DEC-003 has no createIndex privilege, so the schema’s indexes cannot be built by the application; if so, no cluster (test, staging or production) has them unless another user creates them. Nobody has listed the indexes on any cluster, and staging does not exist yet.</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>DEC-003 app role privileges / All environments</t>
+          <t>src/models/RequestHistory.js (unique partial index on actorId, idempotencyKey), DEC-015 §3, M3 API Test Specification S5, DEC-003 civicconnect-app role (inferred cause)</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>None on the code as it stands: the application-level lookup, version check and transition rule each stop the duplicate before the insert. The index is the last line of defence DEC-015 §3 relies on for two requests carrying the same key at the same moment, and on this cluster it is absent or not unique, so that path is unprotected and cannot be tested there.</t>
+          <t>None on the code as it stands: the application-level lookup, version check and transition rule each stop the duplicate before the insert. The index is the last line of defence DEC-015 §3 relies on for two requests carrying the same key at the same moment. On the test cluster it did not act, so that path is unprotected there and cannot be tested there; on staging and production it is unverified (see E24).</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -1657,12 +1657,12 @@
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>Open. Not a release block under the scale (S3). Residual: evidence from this cluster does not show the unique indexes acting.</t>
+          <t>Open. S2: release only with the limitation recorded, unless fixed first. Residual: on the test cluster the unique index on (actorId, idempotencyKey) did not act, so two requests carrying the same key at the same moment are unprotected there; on staging and production this is unverified.</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
-          <t>E. Lindsay</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>
@@ -1683,20 +1683,24 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Unique index on (requestId, requestVersion) fails to build. The app role in DEC-003 has no createIndex privilege, so indexes cannot build on any cluster (test, staging, or production).</t>
+          <t>Observed: on the test cluster, with the version check and the transition rule bypassed (isolated negative verification, case 1), a second requestHistory entry with the same (requestId, requestVersion) was accepted, so the unique index on (requestId, requestVersion) did not act there. Evidence: docs/evidence/M3_API_Negative_Verification.txt. Inferred, not verified: the civicconnect-app role in DEC-003 has no createIndex privilege, so the schema’s indexes cannot be built by the application; if so, no cluster (test, staging or production) has them unless another user creates them. Nobody has listed the indexes on any cluster, and staging does not exist yet.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>DEC-003 app role privileges / All environments</t>
+          <t>src/models/RequestHistory.js (unique index on requestId, requestVersion), DEC-016 decision 4, M3 API Test Specification S5, DEC-003 civicconnect-app role (inferred cause)</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>S3</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="n"/>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>None on the code as it stands: the version check in the service and the version filter in requestRepository.applyChange each stop a second entry for the same version before the insert. The unique index on (requestId, requestVersion) is the last line of defence for two transitions racing on the same version (DEC-016 decision 4); without it, that race could write two history entries with the same requestVersion, which can never be removed (FR-6.7).</t>
+        </is>
+      </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1712,16 +1716,24 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L25" s="5" t="n"/>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="N25" s="5" t="n"/>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Open. S2: release only with the limitation recorded, unless fixed first. Residual: on the test cluster nothing stops two concurrent transitions on the same version from both writing history; on staging and production this is unverified.</t>
+        </is>
+      </c>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t>E. Lindsay</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>
@@ -1737,22 +1749,34 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>E. Lindsay</t>
+          <t>Ethan</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>tests/app.test.js fails intermittently (second flaky test in suite).</t>
+          <t>A second test in the suite fails intermittently. 'health answers without a session, and reports both statuses — AC-NFR-1.6' (tests/app.test.js) failed once, in the NV-56 full-suite run on 2026-10-12, alongside the failure that run was expected to produce. It did not fail in the other nine sabotage runs or in any green re-run in that folder. The failure message was not captured. It was not re-run until it passed; the failure is recorded as it happened, in docs/evidence/M3-client/NV-56_ROLE_value_as_a_quoted_literal.txt and INDEX.txt (PR #89). It is distinct from DEF-013, which is a different test ('login sets __Host-sid…'). Both are in tests/app.test.js, both start the application in-process and call it over HTTP on a loopback port, and both failed during repeated full-suite runs while code was being sabotaged and restored. That points to a common cause in how app.test.js runs its HTTP tests, but it is unconfirmed.</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>tests/app.test.js</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
+          <t>AC-NFR-1.6, tests/app.test.js, npm test and the CI test job; related to DEF-013</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>The test is part of npm test, which is the CI gate. An intermittent failure there means a red build that doesn’t indicate a real fault, and invites re-running until green. Together with DEF-013 it suggests app.test.js’s HTTP tests are not reliable under some condition. Until the cause is known, a failure of either test can’t be told apart from a real fault in the health endpoint or the session cookie.</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1760,19 +1784,27 @@
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L26" s="5" t="n"/>
+          <t>Pending. Capture the failure message, preferably together with DEF-013’s, then decide whether the cause is in the test setup (shared server, ports, timing) or in the application. Fix the cause without weakening any assertion. Until then, every failure is reported as it occurs and never re-run until green.</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="N26" s="5" t="n"/>
+          <t>Pending. Observed on 2026-10-12: 1 failure, in the NV-56 run, out of the full-suite runs made for NV-55 to NV-65. Failure message not captured.</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Not release-blocking (S3). Residual: an intermittent fault in the health endpoint is not ruled out, and the CI gate can go red without a real fault.</t>
+        </is>
+      </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>E. Lindsay</t>
+          <t>Ethan</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add listIndexes refusal observation to DEF-014 and DEF-015
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.2.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.2.xlsx
@@ -1612,7 +1612,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Observed: on the test cluster, with the application-level idempotency lookup bypassed (negative verification, case 2b and the isolated runs), a second requestHistory entry with the same (actorId, idempotencyKey) was accepted, so the unique index on (actorId, idempotencyKey) did not act there. Evidence: docs/evidence/M3_API_Negative_Verification.txt. Inferred, not verified: the civicconnect-app role in DEC-003 has no createIndex privilege, so the schema’s indexes cannot be built by the application; if so, no cluster (test, staging or production) has them unless another user creates them. Nobody has listed the indexes on any cluster, and staging does not exist yet.</t>
+          <t>Observed: on the test cluster, with the application-level idempotency lookup bypassed (negative verification, case 2b and the isolated runs), a second requestHistory entry with the same (actorId, idempotencyKey) was accepted, so the unique index on (actorId, idempotencyKey) did not act there. Evidence: docs/evidence/M3_API_Negative_Verification.txt. Observed (2026-10-12): the civicconnect-app credential is refused listIndexes on every application collection on the test cluster (MongoServerError 8000, AtlasError), so the application cannot list its own indexes; createIndex remains inferred from the role definition. Inferred, not verified: the civicconnect-app role in DEC-003 has no createIndex privilege, so the schema’s indexes cannot be built by the application; if so, no cluster (test, staging or production) has them unless another user creates them. Nobody has listed the indexes on any cluster, and staging does not exist yet.</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Observed: on the test cluster, with the version check and the transition rule bypassed (isolated negative verification, case 1), a second requestHistory entry with the same (requestId, requestVersion) was accepted, so the unique index on (requestId, requestVersion) did not act there. Evidence: docs/evidence/M3_API_Negative_Verification.txt. Inferred, not verified: the civicconnect-app role in DEC-003 has no createIndex privilege, so the schema’s indexes cannot be built by the application; if so, no cluster (test, staging or production) has them unless another user creates them. Nobody has listed the indexes on any cluster, and staging does not exist yet.</t>
+          <t>Observed: on the test cluster, with the version check and the transition rule bypassed (isolated negative verification, case 1), a second requestHistory entry with the same (requestId, requestVersion) was accepted, so the unique index on (requestId, requestVersion) did not act there. Evidence: docs/evidence/M3_API_Negative_Verification.txt. Observed (2026-10-12): the civicconnect-app credential is refused listIndexes on every application collection on the test cluster (MongoServerError 8000, AtlasError), so the application cannot list its own indexes; createIndex remains inferred from the role definition. Inferred, not verified: the civicconnect-app role in DEC-003 has no createIndex privilege, so the schema’s indexes cannot be built by the application; if so, no cluster (test, staging or production) has them unless another user creates them. Nobody has listed the indexes on any cluster, and staging does not exist yet.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">

</xml_diff>